<commit_message>
Restore 849/851 requests for student 106221 (Murphy, Peyton, Gr12)
JC flagged these were incorrectly removed in the bulk Gr12 849/851 removal.
New T2 totals: 6,094 requests, 803 students.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_2_Student_Course_Requests.xlsx
+++ b/templates/Template_2_Student_Course_Requests.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6094"/>
+  <dimension ref="A1:B6096"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="2"/>
@@ -49222,6 +49222,22 @@
         <v>830</v>
       </c>
     </row>
+    <row r="6095">
+      <c r="A6095" t="n">
+        <v>106221</v>
+      </c>
+      <c r="B6095" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6096">
+      <c r="A6096" t="n">
+        <v>106221</v>
+      </c>
+      <c r="B6096" t="n">
+        <v>851</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add missing Theology requests to T2 V3
Added 428 requests: 830×98 (Gr11), 849×165 (Gr12), 851×165 (Gr12)
All grades now have full Theology coverage (0 missing)
New T2 total: 6,528 rows (6,524 unique), 804 students, 143 courses

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_2_Student_Course_Requests.xlsx
+++ b/templates/Template_2_Student_Course_Requests.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6103"/>
+  <dimension ref="A1:B6530"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="11.109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -61493,7 +61493,3430 @@
         </is>
       </c>
     </row>
-    <row r="6103"/>
+    <row r="6103">
+      <c r="A6103" t="n">
+        <v>105477</v>
+      </c>
+      <c r="B6103" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6104">
+      <c r="A6104" t="n">
+        <v>105477</v>
+      </c>
+      <c r="B6104" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6105">
+      <c r="A6105" t="n">
+        <v>106167</v>
+      </c>
+      <c r="B6105" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6106">
+      <c r="A6106" t="n">
+        <v>106167</v>
+      </c>
+      <c r="B6106" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6107">
+      <c r="A6107" t="n">
+        <v>106169</v>
+      </c>
+      <c r="B6107" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6108">
+      <c r="A6108" t="n">
+        <v>106169</v>
+      </c>
+      <c r="B6108" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6109">
+      <c r="A6109" t="n">
+        <v>106170</v>
+      </c>
+      <c r="B6109" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6110">
+      <c r="A6110" t="n">
+        <v>106170</v>
+      </c>
+      <c r="B6110" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6111">
+      <c r="A6111" t="n">
+        <v>106172</v>
+      </c>
+      <c r="B6111" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6112">
+      <c r="A6112" t="n">
+        <v>106172</v>
+      </c>
+      <c r="B6112" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6113">
+      <c r="A6113" t="n">
+        <v>106173</v>
+      </c>
+      <c r="B6113" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6114">
+      <c r="A6114" t="n">
+        <v>106173</v>
+      </c>
+      <c r="B6114" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6115">
+      <c r="A6115" t="n">
+        <v>106174</v>
+      </c>
+      <c r="B6115" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6116">
+      <c r="A6116" t="n">
+        <v>106174</v>
+      </c>
+      <c r="B6116" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6117">
+      <c r="A6117" t="n">
+        <v>106176</v>
+      </c>
+      <c r="B6117" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6118">
+      <c r="A6118" t="n">
+        <v>106176</v>
+      </c>
+      <c r="B6118" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6119">
+      <c r="A6119" t="n">
+        <v>106178</v>
+      </c>
+      <c r="B6119" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6120">
+      <c r="A6120" t="n">
+        <v>106178</v>
+      </c>
+      <c r="B6120" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6121">
+      <c r="A6121" t="n">
+        <v>106182</v>
+      </c>
+      <c r="B6121" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6122">
+      <c r="A6122" t="n">
+        <v>106182</v>
+      </c>
+      <c r="B6122" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6123">
+      <c r="A6123" t="n">
+        <v>106183</v>
+      </c>
+      <c r="B6123" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6124">
+      <c r="A6124" t="n">
+        <v>106183</v>
+      </c>
+      <c r="B6124" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6125">
+      <c r="A6125" t="n">
+        <v>106185</v>
+      </c>
+      <c r="B6125" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6126">
+      <c r="A6126" t="n">
+        <v>106185</v>
+      </c>
+      <c r="B6126" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6127">
+      <c r="A6127" t="n">
+        <v>106186</v>
+      </c>
+      <c r="B6127" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6128">
+      <c r="A6128" t="n">
+        <v>106186</v>
+      </c>
+      <c r="B6128" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6129">
+      <c r="A6129" t="n">
+        <v>106187</v>
+      </c>
+      <c r="B6129" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6130">
+      <c r="A6130" t="n">
+        <v>106187</v>
+      </c>
+      <c r="B6130" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6131">
+      <c r="A6131" t="n">
+        <v>106189</v>
+      </c>
+      <c r="B6131" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6132">
+      <c r="A6132" t="n">
+        <v>106189</v>
+      </c>
+      <c r="B6132" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6133">
+      <c r="A6133" t="n">
+        <v>106192</v>
+      </c>
+      <c r="B6133" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6134">
+      <c r="A6134" t="n">
+        <v>106192</v>
+      </c>
+      <c r="B6134" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6135">
+      <c r="A6135" t="n">
+        <v>106193</v>
+      </c>
+      <c r="B6135" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6136">
+      <c r="A6136" t="n">
+        <v>106193</v>
+      </c>
+      <c r="B6136" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6137">
+      <c r="A6137" t="n">
+        <v>106194</v>
+      </c>
+      <c r="B6137" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6138">
+      <c r="A6138" t="n">
+        <v>106194</v>
+      </c>
+      <c r="B6138" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6139">
+      <c r="A6139" t="n">
+        <v>106195</v>
+      </c>
+      <c r="B6139" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6140">
+      <c r="A6140" t="n">
+        <v>106195</v>
+      </c>
+      <c r="B6140" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6141">
+      <c r="A6141" t="n">
+        <v>106196</v>
+      </c>
+      <c r="B6141" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6142">
+      <c r="A6142" t="n">
+        <v>106196</v>
+      </c>
+      <c r="B6142" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6143">
+      <c r="A6143" t="n">
+        <v>106197</v>
+      </c>
+      <c r="B6143" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6144">
+      <c r="A6144" t="n">
+        <v>106197</v>
+      </c>
+      <c r="B6144" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6145">
+      <c r="A6145" t="n">
+        <v>106199</v>
+      </c>
+      <c r="B6145" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6146">
+      <c r="A6146" t="n">
+        <v>106199</v>
+      </c>
+      <c r="B6146" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6147">
+      <c r="A6147" t="n">
+        <v>106201</v>
+      </c>
+      <c r="B6147" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6148">
+      <c r="A6148" t="n">
+        <v>106201</v>
+      </c>
+      <c r="B6148" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6149">
+      <c r="A6149" t="n">
+        <v>106203</v>
+      </c>
+      <c r="B6149" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6150">
+      <c r="A6150" t="n">
+        <v>106203</v>
+      </c>
+      <c r="B6150" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6151">
+      <c r="A6151" t="n">
+        <v>106204</v>
+      </c>
+      <c r="B6151" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6152">
+      <c r="A6152" t="n">
+        <v>106204</v>
+      </c>
+      <c r="B6152" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6153">
+      <c r="A6153" t="n">
+        <v>106205</v>
+      </c>
+      <c r="B6153" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6154">
+      <c r="A6154" t="n">
+        <v>106205</v>
+      </c>
+      <c r="B6154" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6155">
+      <c r="A6155" t="n">
+        <v>106206</v>
+      </c>
+      <c r="B6155" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6156">
+      <c r="A6156" t="n">
+        <v>106206</v>
+      </c>
+      <c r="B6156" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6157">
+      <c r="A6157" t="n">
+        <v>106208</v>
+      </c>
+      <c r="B6157" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6158">
+      <c r="A6158" t="n">
+        <v>106208</v>
+      </c>
+      <c r="B6158" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6159">
+      <c r="A6159" t="n">
+        <v>106210</v>
+      </c>
+      <c r="B6159" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6160">
+      <c r="A6160" t="n">
+        <v>106210</v>
+      </c>
+      <c r="B6160" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6161">
+      <c r="A6161" t="n">
+        <v>106211</v>
+      </c>
+      <c r="B6161" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6162">
+      <c r="A6162" t="n">
+        <v>106211</v>
+      </c>
+      <c r="B6162" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6163">
+      <c r="A6163" t="n">
+        <v>106212</v>
+      </c>
+      <c r="B6163" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6164">
+      <c r="A6164" t="n">
+        <v>106212</v>
+      </c>
+      <c r="B6164" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6165">
+      <c r="A6165" t="n">
+        <v>106213</v>
+      </c>
+      <c r="B6165" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6166">
+      <c r="A6166" t="n">
+        <v>106213</v>
+      </c>
+      <c r="B6166" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6167">
+      <c r="A6167" t="n">
+        <v>106215</v>
+      </c>
+      <c r="B6167" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6168">
+      <c r="A6168" t="n">
+        <v>106215</v>
+      </c>
+      <c r="B6168" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6169">
+      <c r="A6169" t="n">
+        <v>106216</v>
+      </c>
+      <c r="B6169" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6170">
+      <c r="A6170" t="n">
+        <v>106216</v>
+      </c>
+      <c r="B6170" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6171">
+      <c r="A6171" t="n">
+        <v>106217</v>
+      </c>
+      <c r="B6171" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6172">
+      <c r="A6172" t="n">
+        <v>106217</v>
+      </c>
+      <c r="B6172" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6173">
+      <c r="A6173" t="n">
+        <v>106218</v>
+      </c>
+      <c r="B6173" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6174">
+      <c r="A6174" t="n">
+        <v>106218</v>
+      </c>
+      <c r="B6174" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6175">
+      <c r="A6175" t="n">
+        <v>106219</v>
+      </c>
+      <c r="B6175" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6176">
+      <c r="A6176" t="n">
+        <v>106219</v>
+      </c>
+      <c r="B6176" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6177">
+      <c r="A6177" t="n">
+        <v>106220</v>
+      </c>
+      <c r="B6177" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6178">
+      <c r="A6178" t="n">
+        <v>106220</v>
+      </c>
+      <c r="B6178" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6179">
+      <c r="A6179" t="n">
+        <v>106221</v>
+      </c>
+      <c r="B6179" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6180">
+      <c r="A6180" t="n">
+        <v>106221</v>
+      </c>
+      <c r="B6180" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6181">
+      <c r="A6181" t="n">
+        <v>106222</v>
+      </c>
+      <c r="B6181" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6182">
+      <c r="A6182" t="n">
+        <v>106222</v>
+      </c>
+      <c r="B6182" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6183">
+      <c r="A6183" t="n">
+        <v>106224</v>
+      </c>
+      <c r="B6183" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6184">
+      <c r="A6184" t="n">
+        <v>106224</v>
+      </c>
+      <c r="B6184" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6185">
+      <c r="A6185" t="n">
+        <v>106226</v>
+      </c>
+      <c r="B6185" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6186">
+      <c r="A6186" t="n">
+        <v>106226</v>
+      </c>
+      <c r="B6186" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6187">
+      <c r="A6187" t="n">
+        <v>106227</v>
+      </c>
+      <c r="B6187" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6188">
+      <c r="A6188" t="n">
+        <v>106227</v>
+      </c>
+      <c r="B6188" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6189">
+      <c r="A6189" t="n">
+        <v>106230</v>
+      </c>
+      <c r="B6189" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6190">
+      <c r="A6190" t="n">
+        <v>106230</v>
+      </c>
+      <c r="B6190" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6191">
+      <c r="A6191" t="n">
+        <v>106231</v>
+      </c>
+      <c r="B6191" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6192">
+      <c r="A6192" t="n">
+        <v>106231</v>
+      </c>
+      <c r="B6192" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6193">
+      <c r="A6193" t="n">
+        <v>106232</v>
+      </c>
+      <c r="B6193" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6194">
+      <c r="A6194" t="n">
+        <v>106232</v>
+      </c>
+      <c r="B6194" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6195">
+      <c r="A6195" t="n">
+        <v>106233</v>
+      </c>
+      <c r="B6195" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6196">
+      <c r="A6196" t="n">
+        <v>106233</v>
+      </c>
+      <c r="B6196" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6197">
+      <c r="A6197" t="n">
+        <v>106234</v>
+      </c>
+      <c r="B6197" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6198">
+      <c r="A6198" t="n">
+        <v>106234</v>
+      </c>
+      <c r="B6198" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6199">
+      <c r="A6199" t="n">
+        <v>106235</v>
+      </c>
+      <c r="B6199" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6200">
+      <c r="A6200" t="n">
+        <v>106235</v>
+      </c>
+      <c r="B6200" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6201">
+      <c r="A6201" t="n">
+        <v>106236</v>
+      </c>
+      <c r="B6201" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6202">
+      <c r="A6202" t="n">
+        <v>106236</v>
+      </c>
+      <c r="B6202" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6203">
+      <c r="A6203" t="n">
+        <v>106237</v>
+      </c>
+      <c r="B6203" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6204">
+      <c r="A6204" t="n">
+        <v>106237</v>
+      </c>
+      <c r="B6204" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6205">
+      <c r="A6205" t="n">
+        <v>106238</v>
+      </c>
+      <c r="B6205" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6206">
+      <c r="A6206" t="n">
+        <v>106238</v>
+      </c>
+      <c r="B6206" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6207">
+      <c r="A6207" t="n">
+        <v>106239</v>
+      </c>
+      <c r="B6207" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6208">
+      <c r="A6208" t="n">
+        <v>106239</v>
+      </c>
+      <c r="B6208" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6209">
+      <c r="A6209" t="n">
+        <v>106240</v>
+      </c>
+      <c r="B6209" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6210">
+      <c r="A6210" t="n">
+        <v>106240</v>
+      </c>
+      <c r="B6210" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6211">
+      <c r="A6211" t="n">
+        <v>106241</v>
+      </c>
+      <c r="B6211" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6212">
+      <c r="A6212" t="n">
+        <v>106241</v>
+      </c>
+      <c r="B6212" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6213">
+      <c r="A6213" t="n">
+        <v>106242</v>
+      </c>
+      <c r="B6213" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6214">
+      <c r="A6214" t="n">
+        <v>106242</v>
+      </c>
+      <c r="B6214" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6215">
+      <c r="A6215" t="n">
+        <v>106243</v>
+      </c>
+      <c r="B6215" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6216">
+      <c r="A6216" t="n">
+        <v>106243</v>
+      </c>
+      <c r="B6216" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6217">
+      <c r="A6217" t="n">
+        <v>106244</v>
+      </c>
+      <c r="B6217" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6218">
+      <c r="A6218" t="n">
+        <v>106244</v>
+      </c>
+      <c r="B6218" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6219">
+      <c r="A6219" t="n">
+        <v>106245</v>
+      </c>
+      <c r="B6219" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6220">
+      <c r="A6220" t="n">
+        <v>106245</v>
+      </c>
+      <c r="B6220" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6221">
+      <c r="A6221" t="n">
+        <v>106247</v>
+      </c>
+      <c r="B6221" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6222">
+      <c r="A6222" t="n">
+        <v>106247</v>
+      </c>
+      <c r="B6222" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6223">
+      <c r="A6223" t="n">
+        <v>106248</v>
+      </c>
+      <c r="B6223" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6224">
+      <c r="A6224" t="n">
+        <v>106248</v>
+      </c>
+      <c r="B6224" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6225">
+      <c r="A6225" t="n">
+        <v>106249</v>
+      </c>
+      <c r="B6225" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6226">
+      <c r="A6226" t="n">
+        <v>106249</v>
+      </c>
+      <c r="B6226" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6227">
+      <c r="A6227" t="n">
+        <v>106250</v>
+      </c>
+      <c r="B6227" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6228">
+      <c r="A6228" t="n">
+        <v>106250</v>
+      </c>
+      <c r="B6228" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6229">
+      <c r="A6229" t="n">
+        <v>106251</v>
+      </c>
+      <c r="B6229" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6230">
+      <c r="A6230" t="n">
+        <v>106251</v>
+      </c>
+      <c r="B6230" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6231">
+      <c r="A6231" t="n">
+        <v>106252</v>
+      </c>
+      <c r="B6231" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6232">
+      <c r="A6232" t="n">
+        <v>106252</v>
+      </c>
+      <c r="B6232" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6233">
+      <c r="A6233" t="n">
+        <v>106253</v>
+      </c>
+      <c r="B6233" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6234">
+      <c r="A6234" t="n">
+        <v>106253</v>
+      </c>
+      <c r="B6234" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6235">
+      <c r="A6235" t="n">
+        <v>106254</v>
+      </c>
+      <c r="B6235" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6236">
+      <c r="A6236" t="n">
+        <v>106254</v>
+      </c>
+      <c r="B6236" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6237">
+      <c r="A6237" t="n">
+        <v>106255</v>
+      </c>
+      <c r="B6237" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6238">
+      <c r="A6238" t="n">
+        <v>106255</v>
+      </c>
+      <c r="B6238" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6239">
+      <c r="A6239" t="n">
+        <v>106256</v>
+      </c>
+      <c r="B6239" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6240">
+      <c r="A6240" t="n">
+        <v>106256</v>
+      </c>
+      <c r="B6240" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6241">
+      <c r="A6241" t="n">
+        <v>106257</v>
+      </c>
+      <c r="B6241" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6242">
+      <c r="A6242" t="n">
+        <v>106257</v>
+      </c>
+      <c r="B6242" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6243">
+      <c r="A6243" t="n">
+        <v>106258</v>
+      </c>
+      <c r="B6243" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6244">
+      <c r="A6244" t="n">
+        <v>106258</v>
+      </c>
+      <c r="B6244" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6245">
+      <c r="A6245" t="n">
+        <v>106259</v>
+      </c>
+      <c r="B6245" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6246">
+      <c r="A6246" t="n">
+        <v>106259</v>
+      </c>
+      <c r="B6246" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6247">
+      <c r="A6247" t="n">
+        <v>106260</v>
+      </c>
+      <c r="B6247" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6248">
+      <c r="A6248" t="n">
+        <v>106260</v>
+      </c>
+      <c r="B6248" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6249">
+      <c r="A6249" t="n">
+        <v>106261</v>
+      </c>
+      <c r="B6249" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6250">
+      <c r="A6250" t="n">
+        <v>106261</v>
+      </c>
+      <c r="B6250" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6251">
+      <c r="A6251" t="n">
+        <v>106263</v>
+      </c>
+      <c r="B6251" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6252">
+      <c r="A6252" t="n">
+        <v>106263</v>
+      </c>
+      <c r="B6252" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6253">
+      <c r="A6253" t="n">
+        <v>106264</v>
+      </c>
+      <c r="B6253" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6254">
+      <c r="A6254" t="n">
+        <v>106264</v>
+      </c>
+      <c r="B6254" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6255">
+      <c r="A6255" t="n">
+        <v>106265</v>
+      </c>
+      <c r="B6255" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6256">
+      <c r="A6256" t="n">
+        <v>106265</v>
+      </c>
+      <c r="B6256" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6257">
+      <c r="A6257" t="n">
+        <v>106266</v>
+      </c>
+      <c r="B6257" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6258">
+      <c r="A6258" t="n">
+        <v>106266</v>
+      </c>
+      <c r="B6258" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6259">
+      <c r="A6259" t="n">
+        <v>106267</v>
+      </c>
+      <c r="B6259" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6260">
+      <c r="A6260" t="n">
+        <v>106267</v>
+      </c>
+      <c r="B6260" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6261">
+      <c r="A6261" t="n">
+        <v>106268</v>
+      </c>
+      <c r="B6261" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6262">
+      <c r="A6262" t="n">
+        <v>106268</v>
+      </c>
+      <c r="B6262" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6263">
+      <c r="A6263" t="n">
+        <v>106269</v>
+      </c>
+      <c r="B6263" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6264">
+      <c r="A6264" t="n">
+        <v>106269</v>
+      </c>
+      <c r="B6264" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6265">
+      <c r="A6265" t="n">
+        <v>106270</v>
+      </c>
+      <c r="B6265" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6266">
+      <c r="A6266" t="n">
+        <v>106270</v>
+      </c>
+      <c r="B6266" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6267">
+      <c r="A6267" t="n">
+        <v>106271</v>
+      </c>
+      <c r="B6267" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6268">
+      <c r="A6268" t="n">
+        <v>106271</v>
+      </c>
+      <c r="B6268" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6269">
+      <c r="A6269" t="n">
+        <v>106272</v>
+      </c>
+      <c r="B6269" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6270">
+      <c r="A6270" t="n">
+        <v>106272</v>
+      </c>
+      <c r="B6270" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6271">
+      <c r="A6271" t="n">
+        <v>106273</v>
+      </c>
+      <c r="B6271" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6272">
+      <c r="A6272" t="n">
+        <v>106273</v>
+      </c>
+      <c r="B6272" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6273">
+      <c r="A6273" t="n">
+        <v>106275</v>
+      </c>
+      <c r="B6273" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6274">
+      <c r="A6274" t="n">
+        <v>106275</v>
+      </c>
+      <c r="B6274" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6275">
+      <c r="A6275" t="n">
+        <v>106276</v>
+      </c>
+      <c r="B6275" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6276">
+      <c r="A6276" t="n">
+        <v>106276</v>
+      </c>
+      <c r="B6276" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6277">
+      <c r="A6277" t="n">
+        <v>106277</v>
+      </c>
+      <c r="B6277" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6278">
+      <c r="A6278" t="n">
+        <v>106277</v>
+      </c>
+      <c r="B6278" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6279">
+      <c r="A6279" t="n">
+        <v>106278</v>
+      </c>
+      <c r="B6279" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6280">
+      <c r="A6280" t="n">
+        <v>106278</v>
+      </c>
+      <c r="B6280" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6281">
+      <c r="A6281" t="n">
+        <v>106279</v>
+      </c>
+      <c r="B6281" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6282">
+      <c r="A6282" t="n">
+        <v>106279</v>
+      </c>
+      <c r="B6282" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6283">
+      <c r="A6283" t="n">
+        <v>106280</v>
+      </c>
+      <c r="B6283" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6284">
+      <c r="A6284" t="n">
+        <v>106280</v>
+      </c>
+      <c r="B6284" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6285">
+      <c r="A6285" t="n">
+        <v>106281</v>
+      </c>
+      <c r="B6285" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6286">
+      <c r="A6286" t="n">
+        <v>106281</v>
+      </c>
+      <c r="B6286" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6287">
+      <c r="A6287" t="n">
+        <v>106282</v>
+      </c>
+      <c r="B6287" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6288">
+      <c r="A6288" t="n">
+        <v>106282</v>
+      </c>
+      <c r="B6288" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6289">
+      <c r="A6289" t="n">
+        <v>106283</v>
+      </c>
+      <c r="B6289" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6290">
+      <c r="A6290" t="n">
+        <v>106283</v>
+      </c>
+      <c r="B6290" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6291">
+      <c r="A6291" t="n">
+        <v>106287</v>
+      </c>
+      <c r="B6291" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6292">
+      <c r="A6292" t="n">
+        <v>106287</v>
+      </c>
+      <c r="B6292" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6293">
+      <c r="A6293" t="n">
+        <v>106288</v>
+      </c>
+      <c r="B6293" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6294">
+      <c r="A6294" t="n">
+        <v>106288</v>
+      </c>
+      <c r="B6294" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6295">
+      <c r="A6295" t="n">
+        <v>106289</v>
+      </c>
+      <c r="B6295" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6296">
+      <c r="A6296" t="n">
+        <v>106289</v>
+      </c>
+      <c r="B6296" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6297">
+      <c r="A6297" t="n">
+        <v>106290</v>
+      </c>
+      <c r="B6297" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6298">
+      <c r="A6298" t="n">
+        <v>106290</v>
+      </c>
+      <c r="B6298" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6299">
+      <c r="A6299" t="n">
+        <v>106291</v>
+      </c>
+      <c r="B6299" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6300">
+      <c r="A6300" t="n">
+        <v>106291</v>
+      </c>
+      <c r="B6300" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6301">
+      <c r="A6301" t="n">
+        <v>106292</v>
+      </c>
+      <c r="B6301" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6302">
+      <c r="A6302" t="n">
+        <v>106292</v>
+      </c>
+      <c r="B6302" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6303">
+      <c r="A6303" t="n">
+        <v>106295</v>
+      </c>
+      <c r="B6303" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6304">
+      <c r="A6304" t="n">
+        <v>106295</v>
+      </c>
+      <c r="B6304" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6305">
+      <c r="A6305" t="n">
+        <v>106296</v>
+      </c>
+      <c r="B6305" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6306">
+      <c r="A6306" t="n">
+        <v>106296</v>
+      </c>
+      <c r="B6306" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6307">
+      <c r="A6307" t="n">
+        <v>106297</v>
+      </c>
+      <c r="B6307" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6308">
+      <c r="A6308" t="n">
+        <v>106297</v>
+      </c>
+      <c r="B6308" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6309">
+      <c r="A6309" t="n">
+        <v>106299</v>
+      </c>
+      <c r="B6309" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6310">
+      <c r="A6310" t="n">
+        <v>106299</v>
+      </c>
+      <c r="B6310" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6311">
+      <c r="A6311" t="n">
+        <v>106300</v>
+      </c>
+      <c r="B6311" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6312">
+      <c r="A6312" t="n">
+        <v>106300</v>
+      </c>
+      <c r="B6312" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6313">
+      <c r="A6313" t="n">
+        <v>106301</v>
+      </c>
+      <c r="B6313" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6314">
+      <c r="A6314" t="n">
+        <v>106301</v>
+      </c>
+      <c r="B6314" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6315">
+      <c r="A6315" t="n">
+        <v>106303</v>
+      </c>
+      <c r="B6315" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6316">
+      <c r="A6316" t="n">
+        <v>106303</v>
+      </c>
+      <c r="B6316" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6317">
+      <c r="A6317" t="n">
+        <v>106306</v>
+      </c>
+      <c r="B6317" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6318">
+      <c r="A6318" t="n">
+        <v>106306</v>
+      </c>
+      <c r="B6318" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6319">
+      <c r="A6319" t="n">
+        <v>106307</v>
+      </c>
+      <c r="B6319" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6320">
+      <c r="A6320" t="n">
+        <v>106307</v>
+      </c>
+      <c r="B6320" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6321">
+      <c r="A6321" t="n">
+        <v>106308</v>
+      </c>
+      <c r="B6321" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6322">
+      <c r="A6322" t="n">
+        <v>106308</v>
+      </c>
+      <c r="B6322" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6323">
+      <c r="A6323" t="n">
+        <v>106309</v>
+      </c>
+      <c r="B6323" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6324">
+      <c r="A6324" t="n">
+        <v>106309</v>
+      </c>
+      <c r="B6324" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6325">
+      <c r="A6325" t="n">
+        <v>106310</v>
+      </c>
+      <c r="B6325" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6326">
+      <c r="A6326" t="n">
+        <v>106310</v>
+      </c>
+      <c r="B6326" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6327">
+      <c r="A6327" t="n">
+        <v>106311</v>
+      </c>
+      <c r="B6327" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6328">
+      <c r="A6328" t="n">
+        <v>106311</v>
+      </c>
+      <c r="B6328" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6329">
+      <c r="A6329" t="n">
+        <v>106312</v>
+      </c>
+      <c r="B6329" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6330">
+      <c r="A6330" t="n">
+        <v>106312</v>
+      </c>
+      <c r="B6330" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6331">
+      <c r="A6331" t="n">
+        <v>106313</v>
+      </c>
+      <c r="B6331" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6332">
+      <c r="A6332" t="n">
+        <v>106313</v>
+      </c>
+      <c r="B6332" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6333">
+      <c r="A6333" t="n">
+        <v>106314</v>
+      </c>
+      <c r="B6333" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6334">
+      <c r="A6334" t="n">
+        <v>106314</v>
+      </c>
+      <c r="B6334" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6335">
+      <c r="A6335" t="n">
+        <v>106316</v>
+      </c>
+      <c r="B6335" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6336">
+      <c r="A6336" t="n">
+        <v>106316</v>
+      </c>
+      <c r="B6336" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6337">
+      <c r="A6337" t="n">
+        <v>106322</v>
+      </c>
+      <c r="B6337" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6338">
+      <c r="A6338" t="n">
+        <v>106322</v>
+      </c>
+      <c r="B6338" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6339">
+      <c r="A6339" t="n">
+        <v>106323</v>
+      </c>
+      <c r="B6339" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6340">
+      <c r="A6340" t="n">
+        <v>106323</v>
+      </c>
+      <c r="B6340" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6341">
+      <c r="A6341" t="n">
+        <v>106324</v>
+      </c>
+      <c r="B6341" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6342">
+      <c r="A6342" t="n">
+        <v>106324</v>
+      </c>
+      <c r="B6342" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6343">
+      <c r="A6343" t="n">
+        <v>106325</v>
+      </c>
+      <c r="B6343" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6344">
+      <c r="A6344" t="n">
+        <v>106325</v>
+      </c>
+      <c r="B6344" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6345">
+      <c r="A6345" t="n">
+        <v>106332</v>
+      </c>
+      <c r="B6345" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6346">
+      <c r="A6346" t="n">
+        <v>106332</v>
+      </c>
+      <c r="B6346" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6347">
+      <c r="A6347" t="n">
+        <v>106333</v>
+      </c>
+      <c r="B6347" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6348">
+      <c r="A6348" t="n">
+        <v>106333</v>
+      </c>
+      <c r="B6348" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6349">
+      <c r="A6349" t="n">
+        <v>106334</v>
+      </c>
+      <c r="B6349" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6350">
+      <c r="A6350" t="n">
+        <v>106334</v>
+      </c>
+      <c r="B6350" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6351">
+      <c r="A6351" t="n">
+        <v>106335</v>
+      </c>
+      <c r="B6351" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6352">
+      <c r="A6352" t="n">
+        <v>106335</v>
+      </c>
+      <c r="B6352" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6353">
+      <c r="A6353" t="n">
+        <v>106336</v>
+      </c>
+      <c r="B6353" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6354">
+      <c r="A6354" t="n">
+        <v>106336</v>
+      </c>
+      <c r="B6354" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6355">
+      <c r="A6355" t="n">
+        <v>106337</v>
+      </c>
+      <c r="B6355" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6356">
+      <c r="A6356" t="n">
+        <v>106337</v>
+      </c>
+      <c r="B6356" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6357">
+      <c r="A6357" t="n">
+        <v>106341</v>
+      </c>
+      <c r="B6357" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6358">
+      <c r="A6358" t="n">
+        <v>106341</v>
+      </c>
+      <c r="B6358" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6359">
+      <c r="A6359" t="n">
+        <v>106344</v>
+      </c>
+      <c r="B6359" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6360">
+      <c r="A6360" t="n">
+        <v>106344</v>
+      </c>
+      <c r="B6360" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6361">
+      <c r="A6361" t="n">
+        <v>106347</v>
+      </c>
+      <c r="B6361" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6362">
+      <c r="A6362" t="n">
+        <v>106347</v>
+      </c>
+      <c r="B6362" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6363">
+      <c r="A6363" t="n">
+        <v>106349</v>
+      </c>
+      <c r="B6363" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6364">
+      <c r="A6364" t="n">
+        <v>106349</v>
+      </c>
+      <c r="B6364" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6365">
+      <c r="A6365" t="n">
+        <v>106350</v>
+      </c>
+      <c r="B6365" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6366">
+      <c r="A6366" t="n">
+        <v>106350</v>
+      </c>
+      <c r="B6366" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6367">
+      <c r="A6367" t="n">
+        <v>106351</v>
+      </c>
+      <c r="B6367" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6368">
+      <c r="A6368" t="n">
+        <v>106351</v>
+      </c>
+      <c r="B6368" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6369">
+      <c r="A6369" t="n">
+        <v>106353</v>
+      </c>
+      <c r="B6369" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6370">
+      <c r="A6370" t="n">
+        <v>106353</v>
+      </c>
+      <c r="B6370" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6371">
+      <c r="A6371" t="n">
+        <v>106356</v>
+      </c>
+      <c r="B6371" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6372">
+      <c r="A6372" t="n">
+        <v>106356</v>
+      </c>
+      <c r="B6372" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6373">
+      <c r="A6373" t="n">
+        <v>106357</v>
+      </c>
+      <c r="B6373" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6374">
+      <c r="A6374" t="n">
+        <v>106357</v>
+      </c>
+      <c r="B6374" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6375">
+      <c r="A6375" t="n">
+        <v>106736</v>
+      </c>
+      <c r="B6375" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6376">
+      <c r="A6376" t="n">
+        <v>106736</v>
+      </c>
+      <c r="B6376" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6377">
+      <c r="A6377" t="n">
+        <v>106739</v>
+      </c>
+      <c r="B6377" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6378">
+      <c r="A6378" t="n">
+        <v>106739</v>
+      </c>
+      <c r="B6378" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6379">
+      <c r="A6379" t="n">
+        <v>107008</v>
+      </c>
+      <c r="B6379" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6380">
+      <c r="A6380" t="n">
+        <v>107008</v>
+      </c>
+      <c r="B6380" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6381">
+      <c r="A6381" t="n">
+        <v>107127</v>
+      </c>
+      <c r="B6381" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6382">
+      <c r="A6382" t="n">
+        <v>107127</v>
+      </c>
+      <c r="B6382" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6383">
+      <c r="A6383" t="n">
+        <v>107254</v>
+      </c>
+      <c r="B6383" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6384">
+      <c r="A6384" t="n">
+        <v>107254</v>
+      </c>
+      <c r="B6384" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6385">
+      <c r="A6385" t="n">
+        <v>107376</v>
+      </c>
+      <c r="B6385" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6386">
+      <c r="A6386" t="n">
+        <v>107376</v>
+      </c>
+      <c r="B6386" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6387">
+      <c r="A6387" t="n">
+        <v>108291</v>
+      </c>
+      <c r="B6387" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6388">
+      <c r="A6388" t="n">
+        <v>108293</v>
+      </c>
+      <c r="B6388" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6389">
+      <c r="A6389" t="n">
+        <v>108298</v>
+      </c>
+      <c r="B6389" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6390">
+      <c r="A6390" t="n">
+        <v>108309</v>
+      </c>
+      <c r="B6390" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6391">
+      <c r="A6391" t="n">
+        <v>108326</v>
+      </c>
+      <c r="B6391" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6392">
+      <c r="A6392" t="n">
+        <v>108361</v>
+      </c>
+      <c r="B6392" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6393">
+      <c r="A6393" t="n">
+        <v>108368</v>
+      </c>
+      <c r="B6393" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6394">
+      <c r="A6394" t="n">
+        <v>108382</v>
+      </c>
+      <c r="B6394" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6395">
+      <c r="A6395" t="n">
+        <v>108388</v>
+      </c>
+      <c r="B6395" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6396">
+      <c r="A6396" t="n">
+        <v>108402</v>
+      </c>
+      <c r="B6396" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6397">
+      <c r="A6397" t="n">
+        <v>108404</v>
+      </c>
+      <c r="B6397" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6398">
+      <c r="A6398" t="n">
+        <v>108408</v>
+      </c>
+      <c r="B6398" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6399">
+      <c r="A6399" t="n">
+        <v>108437</v>
+      </c>
+      <c r="B6399" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6400">
+      <c r="A6400" t="n">
+        <v>108479</v>
+      </c>
+      <c r="B6400" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6401">
+      <c r="A6401" t="n">
+        <v>108482</v>
+      </c>
+      <c r="B6401" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6402">
+      <c r="A6402" t="n">
+        <v>108507</v>
+      </c>
+      <c r="B6402" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6403">
+      <c r="A6403" t="n">
+        <v>108568</v>
+      </c>
+      <c r="B6403" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6404">
+      <c r="A6404" t="n">
+        <v>108571</v>
+      </c>
+      <c r="B6404" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6405">
+      <c r="A6405" t="n">
+        <v>108592</v>
+      </c>
+      <c r="B6405" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6406">
+      <c r="A6406" t="n">
+        <v>108605</v>
+      </c>
+      <c r="B6406" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6407">
+      <c r="A6407" t="n">
+        <v>108608</v>
+      </c>
+      <c r="B6407" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6408">
+      <c r="A6408" t="n">
+        <v>108615</v>
+      </c>
+      <c r="B6408" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6409">
+      <c r="A6409" t="n">
+        <v>108622</v>
+      </c>
+      <c r="B6409" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6410">
+      <c r="A6410" t="n">
+        <v>108658</v>
+      </c>
+      <c r="B6410" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6411">
+      <c r="A6411" t="n">
+        <v>108666</v>
+      </c>
+      <c r="B6411" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6412">
+      <c r="A6412" t="n">
+        <v>108673</v>
+      </c>
+      <c r="B6412" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6413">
+      <c r="A6413" t="n">
+        <v>108734</v>
+      </c>
+      <c r="B6413" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6414">
+      <c r="A6414" t="n">
+        <v>108738</v>
+      </c>
+      <c r="B6414" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6415">
+      <c r="A6415" t="n">
+        <v>108756</v>
+      </c>
+      <c r="B6415" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6416">
+      <c r="A6416" t="n">
+        <v>108756</v>
+      </c>
+      <c r="B6416" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6417">
+      <c r="A6417" t="n">
+        <v>108772</v>
+      </c>
+      <c r="B6417" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6418">
+      <c r="A6418" t="n">
+        <v>108803</v>
+      </c>
+      <c r="B6418" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6419">
+      <c r="A6419" t="n">
+        <v>108808</v>
+      </c>
+      <c r="B6419" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6420">
+      <c r="A6420" t="n">
+        <v>108813</v>
+      </c>
+      <c r="B6420" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6421">
+      <c r="A6421" t="n">
+        <v>108828</v>
+      </c>
+      <c r="B6421" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6422">
+      <c r="A6422" t="n">
+        <v>108870</v>
+      </c>
+      <c r="B6422" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6423">
+      <c r="A6423" t="n">
+        <v>108935</v>
+      </c>
+      <c r="B6423" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6424">
+      <c r="A6424" t="n">
+        <v>108938</v>
+      </c>
+      <c r="B6424" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6425">
+      <c r="A6425" t="n">
+        <v>108962</v>
+      </c>
+      <c r="B6425" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6426">
+      <c r="A6426" t="n">
+        <v>108989</v>
+      </c>
+      <c r="B6426" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6427">
+      <c r="A6427" t="n">
+        <v>109005</v>
+      </c>
+      <c r="B6427" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6428">
+      <c r="A6428" t="n">
+        <v>109026</v>
+      </c>
+      <c r="B6428" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6429">
+      <c r="A6429" t="n">
+        <v>109182</v>
+      </c>
+      <c r="B6429" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6430">
+      <c r="A6430" t="n">
+        <v>109204</v>
+      </c>
+      <c r="B6430" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6431">
+      <c r="A6431" t="n">
+        <v>109211</v>
+      </c>
+      <c r="B6431" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6432">
+      <c r="A6432" t="n">
+        <v>109214</v>
+      </c>
+      <c r="B6432" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6433">
+      <c r="A6433" t="n">
+        <v>109421</v>
+      </c>
+      <c r="B6433" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6434">
+      <c r="A6434" t="n">
+        <v>109435</v>
+      </c>
+      <c r="B6434" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6435">
+      <c r="A6435" t="n">
+        <v>109453</v>
+      </c>
+      <c r="B6435" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6436">
+      <c r="A6436" t="n">
+        <v>109471</v>
+      </c>
+      <c r="B6436" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6437">
+      <c r="A6437" t="n">
+        <v>109511</v>
+      </c>
+      <c r="B6437" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6438">
+      <c r="A6438" t="n">
+        <v>109520</v>
+      </c>
+      <c r="B6438" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6439">
+      <c r="A6439" t="n">
+        <v>109554</v>
+      </c>
+      <c r="B6439" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6440">
+      <c r="A6440" t="n">
+        <v>109580</v>
+      </c>
+      <c r="B6440" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6441">
+      <c r="A6441" t="n">
+        <v>109583</v>
+      </c>
+      <c r="B6441" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6442">
+      <c r="A6442" t="n">
+        <v>109592</v>
+      </c>
+      <c r="B6442" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6443">
+      <c r="A6443" t="n">
+        <v>109726</v>
+      </c>
+      <c r="B6443" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6444">
+      <c r="A6444" t="n">
+        <v>109738</v>
+      </c>
+      <c r="B6444" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6445">
+      <c r="A6445" t="n">
+        <v>109753</v>
+      </c>
+      <c r="B6445" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6446">
+      <c r="A6446" t="n">
+        <v>109824</v>
+      </c>
+      <c r="B6446" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6447">
+      <c r="A6447" t="n">
+        <v>109833</v>
+      </c>
+      <c r="B6447" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6448">
+      <c r="A6448" t="n">
+        <v>109845</v>
+      </c>
+      <c r="B6448" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6449">
+      <c r="A6449" t="n">
+        <v>110097</v>
+      </c>
+      <c r="B6449" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6450">
+      <c r="A6450" t="n">
+        <v>110098</v>
+      </c>
+      <c r="B6450" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6451">
+      <c r="A6451" t="n">
+        <v>110101</v>
+      </c>
+      <c r="B6451" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6452">
+      <c r="A6452" t="n">
+        <v>110133</v>
+      </c>
+      <c r="B6452" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6453">
+      <c r="A6453" t="n">
+        <v>110274</v>
+      </c>
+      <c r="B6453" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6454">
+      <c r="A6454" t="n">
+        <v>110377</v>
+      </c>
+      <c r="B6454" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6455">
+      <c r="A6455" t="n">
+        <v>110396</v>
+      </c>
+      <c r="B6455" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6456">
+      <c r="A6456" t="n">
+        <v>110478</v>
+      </c>
+      <c r="B6456" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6457">
+      <c r="A6457" t="n">
+        <v>110478</v>
+      </c>
+      <c r="B6457" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6458">
+      <c r="A6458" t="n">
+        <v>110767</v>
+      </c>
+      <c r="B6458" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6459">
+      <c r="A6459" t="n">
+        <v>110886</v>
+      </c>
+      <c r="B6459" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6460">
+      <c r="A6460" t="n">
+        <v>110886</v>
+      </c>
+      <c r="B6460" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6461">
+      <c r="A6461" t="n">
+        <v>111057</v>
+      </c>
+      <c r="B6461" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6462">
+      <c r="A6462" t="n">
+        <v>111267</v>
+      </c>
+      <c r="B6462" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6463">
+      <c r="A6463" t="n">
+        <v>111356</v>
+      </c>
+      <c r="B6463" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6464">
+      <c r="A6464" t="n">
+        <v>111725</v>
+      </c>
+      <c r="B6464" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6465">
+      <c r="A6465" t="n">
+        <v>111725</v>
+      </c>
+      <c r="B6465" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6466">
+      <c r="A6466" t="n">
+        <v>111766</v>
+      </c>
+      <c r="B6466" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6467">
+      <c r="A6467" t="n">
+        <v>111831</v>
+      </c>
+      <c r="B6467" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6468">
+      <c r="A6468" t="n">
+        <v>111831</v>
+      </c>
+      <c r="B6468" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6469">
+      <c r="A6469" t="n">
+        <v>111850</v>
+      </c>
+      <c r="B6469" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6470">
+      <c r="A6470" t="n">
+        <v>111850</v>
+      </c>
+      <c r="B6470" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6471">
+      <c r="A6471" t="n">
+        <v>111916</v>
+      </c>
+      <c r="B6471" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6472">
+      <c r="A6472" t="n">
+        <v>111947</v>
+      </c>
+      <c r="B6472" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6473">
+      <c r="A6473" t="n">
+        <v>112020</v>
+      </c>
+      <c r="B6473" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6474">
+      <c r="A6474" t="n">
+        <v>112051</v>
+      </c>
+      <c r="B6474" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6475">
+      <c r="A6475" t="n">
+        <v>112051</v>
+      </c>
+      <c r="B6475" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6476">
+      <c r="A6476" t="n">
+        <v>112088</v>
+      </c>
+      <c r="B6476" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6477">
+      <c r="A6477" t="n">
+        <v>112088</v>
+      </c>
+      <c r="B6477" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6478">
+      <c r="A6478" t="n">
+        <v>112275</v>
+      </c>
+      <c r="B6478" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6479">
+      <c r="A6479" t="n">
+        <v>112306</v>
+      </c>
+      <c r="B6479" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6480">
+      <c r="A6480" t="n">
+        <v>112306</v>
+      </c>
+      <c r="B6480" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6481">
+      <c r="A6481" t="n">
+        <v>112468</v>
+      </c>
+      <c r="B6481" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6482">
+      <c r="A6482" t="n">
+        <v>112468</v>
+      </c>
+      <c r="B6482" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6483">
+      <c r="A6483" t="n">
+        <v>112950</v>
+      </c>
+      <c r="B6483" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6484">
+      <c r="A6484" t="n">
+        <v>113199</v>
+      </c>
+      <c r="B6484" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6485">
+      <c r="A6485" t="n">
+        <v>113761</v>
+      </c>
+      <c r="B6485" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6486">
+      <c r="A6486" t="n">
+        <v>113761</v>
+      </c>
+      <c r="B6486" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6487">
+      <c r="A6487" t="n">
+        <v>113957</v>
+      </c>
+      <c r="B6487" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6488">
+      <c r="A6488" t="n">
+        <v>113957</v>
+      </c>
+      <c r="B6488" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6489">
+      <c r="A6489" t="n">
+        <v>114156</v>
+      </c>
+      <c r="B6489" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6490">
+      <c r="A6490" t="n">
+        <v>115627</v>
+      </c>
+      <c r="B6490" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6491">
+      <c r="A6491" t="n">
+        <v>115627</v>
+      </c>
+      <c r="B6491" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6492">
+      <c r="A6492" t="n">
+        <v>115730</v>
+      </c>
+      <c r="B6492" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6493">
+      <c r="A6493" t="n">
+        <v>115730</v>
+      </c>
+      <c r="B6493" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6494">
+      <c r="A6494" t="n">
+        <v>115797</v>
+      </c>
+      <c r="B6494" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6495">
+      <c r="A6495" t="n">
+        <v>115797</v>
+      </c>
+      <c r="B6495" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6496">
+      <c r="A6496" t="n">
+        <v>116044</v>
+      </c>
+      <c r="B6496" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6497">
+      <c r="A6497" t="n">
+        <v>116044</v>
+      </c>
+      <c r="B6497" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6498">
+      <c r="A6498" t="n">
+        <v>116149</v>
+      </c>
+      <c r="B6498" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6499">
+      <c r="A6499" t="n">
+        <v>116201</v>
+      </c>
+      <c r="B6499" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6500">
+      <c r="A6500" t="n">
+        <v>116628</v>
+      </c>
+      <c r="B6500" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6501">
+      <c r="A6501" t="n">
+        <v>116628</v>
+      </c>
+      <c r="B6501" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6502">
+      <c r="A6502" t="n">
+        <v>116815</v>
+      </c>
+      <c r="B6502" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6503">
+      <c r="A6503" t="n">
+        <v>116892</v>
+      </c>
+      <c r="B6503" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6504">
+      <c r="A6504" t="n">
+        <v>116980</v>
+      </c>
+      <c r="B6504" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6505">
+      <c r="A6505" t="n">
+        <v>117105</v>
+      </c>
+      <c r="B6505" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6506">
+      <c r="A6506" t="n">
+        <v>117132</v>
+      </c>
+      <c r="B6506" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6507">
+      <c r="A6507" t="n">
+        <v>117132</v>
+      </c>
+      <c r="B6507" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6508">
+      <c r="A6508" t="n">
+        <v>117153</v>
+      </c>
+      <c r="B6508" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6509">
+      <c r="A6509" t="n">
+        <v>117239</v>
+      </c>
+      <c r="B6509" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6510">
+      <c r="A6510" t="n">
+        <v>117239</v>
+      </c>
+      <c r="B6510" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6511">
+      <c r="A6511" t="n">
+        <v>117247</v>
+      </c>
+      <c r="B6511" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6512">
+      <c r="A6512" t="n">
+        <v>117247</v>
+      </c>
+      <c r="B6512" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6513">
+      <c r="A6513" t="n">
+        <v>117392</v>
+      </c>
+      <c r="B6513" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6514">
+      <c r="A6514" t="n">
+        <v>118186</v>
+      </c>
+      <c r="B6514" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6515">
+      <c r="A6515" t="n">
+        <v>118186</v>
+      </c>
+      <c r="B6515" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6516">
+      <c r="A6516" t="n">
+        <v>118420</v>
+      </c>
+      <c r="B6516" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6517">
+      <c r="A6517" t="n">
+        <v>119012</v>
+      </c>
+      <c r="B6517" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6518">
+      <c r="A6518" t="n">
+        <v>119400</v>
+      </c>
+      <c r="B6518" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6519">
+      <c r="A6519" t="n">
+        <v>119400</v>
+      </c>
+      <c r="B6519" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6520">
+      <c r="A6520" t="n">
+        <v>119514</v>
+      </c>
+      <c r="B6520" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6521">
+      <c r="A6521" t="n">
+        <v>119656</v>
+      </c>
+      <c r="B6521" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6522">
+      <c r="A6522" t="n">
+        <v>119659</v>
+      </c>
+      <c r="B6522" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6523">
+      <c r="A6523" t="n">
+        <v>120546</v>
+      </c>
+      <c r="B6523" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6524">
+      <c r="A6524" t="n">
+        <v>121187</v>
+      </c>
+      <c r="B6524" t="n">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="6525">
+      <c r="A6525" t="n">
+        <v>121187</v>
+      </c>
+      <c r="B6525" t="n">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6526">
+      <c r="A6526" t="n">
+        <v>121320</v>
+      </c>
+      <c r="B6526" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6527">
+      <c r="A6527" t="n">
+        <v>121384</v>
+      </c>
+      <c r="B6527" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6528">
+      <c r="A6528" t="n">
+        <v>121441</v>
+      </c>
+      <c r="B6528" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6529">
+      <c r="A6529" t="n">
+        <v>121949</v>
+      </c>
+      <c r="B6529" t="n">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="6530">
+      <c r="A6530" t="n">
+        <v>121986</v>
+      </c>
+      <c r="B6530" t="n">
+        <v>830</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>